<commit_message>
Pushed modified MDPI_Tibet Database to accommodate for error on parsing
</commit_message>
<xml_diff>
--- a/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1.1_Data-Acquisition-Wrapper/Zwischenstände/MDPI_Tibet_Datenbank/after_conversion_mdpi_tibet_mapped_readable.xlsx
+++ b/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1.1_Data-Acquisition-Wrapper/Zwischenstände/MDPI_Tibet_Datenbank/after_conversion_mdpi_tibet_mapped_readable.xlsx
@@ -517,7 +517,7 @@
     <col min="7" max="7" width="22.7109375" customWidth="1"/>
     <col min="8" max="8" width="18.7109375" customWidth="1"/>
     <col min="9" max="9" width="38.7109375" customWidth="1"/>
-    <col min="10" max="10" width="7.7109375" customWidth="1"/>
+    <col min="10" max="10" width="6.7109375" customWidth="1"/>
     <col min="11" max="11" width="23.7109375" customWidth="1"/>
     <col min="12" max="12" width="34.7109375" customWidth="1"/>
     <col min="13" max="13" width="14.7109375" customWidth="1"/>
@@ -900,7 +900,7 @@
         <v>8.24</v>
       </c>
       <c r="L6">
-        <v>15.76651471811327</v>
+        <v>26.0441969630032</v>
       </c>
       <c r="N6">
         <v>10.1071045994416</v>
@@ -918,7 +918,7 @@
         <v>1.579013116801999</v>
       </c>
       <c r="S6">
-        <v>0.0116151289480929</v>
+        <v>10.28929737383802</v>
       </c>
       <c r="U6">
         <v>0.8900642738942612</v>
@@ -959,7 +959,7 @@
         <v>8.24</v>
       </c>
       <c r="L7">
-        <v>14.01676797810735</v>
+        <v>23.55780630711544</v>
       </c>
       <c r="N7">
         <v>11.4811940911629</v>
@@ -974,7 +974,10 @@
         <v>0.4211565585331452</v>
       </c>
       <c r="R7">
-        <v>0.0448677909639808</v>
+        <v>0</v>
+      </c>
+      <c r="S7">
+        <v>9.516395484522294</v>
       </c>
       <c r="U7">
         <v>0.2225160684735653</v>
@@ -983,7 +986,7 @@
         <v>221.0759027266028</v>
       </c>
       <c r="AA7">
-        <v>0</v>
+        <v>0.0695106354497789</v>
       </c>
       <c r="AD7">
         <v>1</v>
@@ -1251,7 +1254,7 @@
         <v>8.24</v>
       </c>
       <c r="L12">
-        <v>15.33945686688352</v>
+        <v>25.83197695971041</v>
       </c>
       <c r="N12">
         <v>9.133628093435824</v>
@@ -1268,6 +1271,9 @@
       <c r="R12">
         <v>1.559442015407037</v>
       </c>
+      <c r="S12">
+        <v>10.49252009282689</v>
+      </c>
       <c r="T12">
         <v>0.1649855907780979</v>
       </c>
@@ -1567,7 +1573,7 @@
         <v>6.91</v>
       </c>
       <c r="L17">
-        <v>18.48176705297896</v>
+        <v>18.4703342952453</v>
       </c>
       <c r="N17">
         <v>12.78786228778549</v>
@@ -1584,6 +1590,9 @@
       <c r="R17">
         <v>2.188007495315428</v>
       </c>
+      <c r="S17">
+        <v>0</v>
+      </c>
       <c r="U17">
         <v>1.133041590043557</v>
       </c>
@@ -1591,7 +1600,7 @@
         <v>357.9324139383093</v>
       </c>
       <c r="AA17">
-        <v>0.0114327577336629</v>
+        <v>0</v>
       </c>
       <c r="AD17">
         <v>1</v>
@@ -1989,7 +1998,7 @@
         <v>8.130000000000001</v>
       </c>
       <c r="L24">
-        <v>15.84833630672409</v>
+        <v>15.91133866081134</v>
       </c>
       <c r="N24">
         <v>7.211903695074101</v>
@@ -2006,6 +2015,9 @@
       <c r="R24">
         <v>2.487091401207579</v>
       </c>
+      <c r="S24">
+        <v>3.95350133078103</v>
+      </c>
       <c r="U24">
         <v>0.457820416744462</v>
       </c>
@@ -2013,7 +2025,7 @@
         <v>358.9851563322455</v>
       </c>
       <c r="AA24">
-        <v>3.890498976693777</v>
+        <v>0</v>
       </c>
       <c r="AD24">
         <v>1</v>
@@ -2659,7 +2671,7 @@
         <v>7.4</v>
       </c>
       <c r="L35">
-        <v>27.1419163497648</v>
+        <v>27.28730780396549</v>
       </c>
       <c r="N35">
         <v>11.93313425637291</v>
@@ -2676,6 +2688,9 @@
       <c r="R35">
         <v>3.172912762856548</v>
       </c>
+      <c r="S35">
+        <v>9.123552857573651</v>
+      </c>
       <c r="U35">
         <v>0.4798162579958719</v>
       </c>
@@ -2683,7 +2698,7 @@
         <v>353.1950731655963</v>
       </c>
       <c r="AA35">
-        <v>8.97816140337296</v>
+        <v>0</v>
       </c>
       <c r="AD35">
         <v>1</v>
@@ -3122,40 +3137,52 @@
         <v>39</v>
       </c>
       <c r="C43">
-        <v>3.87</v>
+        <v>25.5621</v>
       </c>
       <c r="D43">
-        <v>92.16</v>
+        <v>100.1299</v>
       </c>
       <c r="F43" t="s">
         <v>42</v>
       </c>
       <c r="H43">
-        <v>1</v>
+        <v>63</v>
       </c>
       <c r="I43">
-        <v>5.19</v>
+        <v>471</v>
       </c>
       <c r="J43">
-        <v>10.98</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="L43">
-        <v>10.55644457807197</v>
+        <v>8.252648200904737</v>
       </c>
       <c r="N43">
-        <v>0.1874746979841337</v>
+        <v>4.008739713739621</v>
       </c>
       <c r="O43">
+        <v>0.0411437975725159</v>
+      </c>
+      <c r="P43">
+        <v>0.2739657667548281</v>
+      </c>
+      <c r="Q43">
+        <v>0.1215796897038081</v>
+      </c>
+      <c r="R43">
+        <v>0.8790339371226317</v>
+      </c>
+      <c r="S43">
+        <v>2.556017359153544</v>
+      </c>
+      <c r="U43">
+        <v>0.09898128563134451</v>
+      </c>
+      <c r="Z43">
+        <v>273.1866512264449</v>
+      </c>
+      <c r="AA43">
         <v>0</v>
-      </c>
-      <c r="P43">
-        <v>0</v>
-      </c>
-      <c r="U43">
-        <v>2.159684692173317</v>
-      </c>
-      <c r="Z43">
-        <v>8209.285187914516</v>
       </c>
       <c r="AD43">
         <v>1</v>
@@ -3169,40 +3196,52 @@
         <v>39</v>
       </c>
       <c r="C44">
-        <v>3.85</v>
+        <v>25.5621</v>
       </c>
       <c r="D44">
-        <v>96.59999999999999</v>
+        <v>100.1299</v>
       </c>
       <c r="F44" t="s">
         <v>42</v>
       </c>
       <c r="H44">
-        <v>0.99</v>
+        <v>63</v>
       </c>
       <c r="I44">
-        <v>6.21</v>
+        <v>471</v>
       </c>
       <c r="J44">
-        <v>12.93</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="L44">
-        <v>12.1811049990346</v>
+        <v>9.04752650992269</v>
       </c>
       <c r="N44">
-        <v>0.1635510126265296</v>
+        <v>4.201869100990097</v>
       </c>
       <c r="O44">
-        <v>0.0785846533635054</v>
+        <v>0.0407323595967907</v>
       </c>
       <c r="P44">
-        <v>0</v>
+        <v>0.3226208892659314</v>
+      </c>
+      <c r="Q44">
+        <v>0.1060648801128349</v>
+      </c>
+      <c r="R44">
+        <v>0.8628981886321049</v>
+      </c>
+      <c r="S44">
+        <v>3.057190806466416</v>
       </c>
       <c r="U44">
-        <v>2.12004102480159</v>
+        <v>0.0984697544394513</v>
       </c>
       <c r="Z44">
-        <v>9818.928308242972</v>
+        <v>326.8765133171913</v>
+      </c>
+      <c r="AA44">
+        <v>0.0308040171018742</v>
       </c>
       <c r="AD44">
         <v>1</v>
@@ -3216,40 +3255,52 @@
         <v>39</v>
       </c>
       <c r="C45">
-        <v>3.45</v>
+        <v>25.5621</v>
       </c>
       <c r="D45">
-        <v>92.95999999999999</v>
+        <v>100.1299</v>
       </c>
       <c r="F45" t="s">
         <v>42</v>
       </c>
       <c r="H45">
-        <v>1.07</v>
+        <v>63</v>
       </c>
       <c r="I45">
-        <v>5.81</v>
+        <v>471</v>
       </c>
       <c r="J45">
-        <v>12.63</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="L45">
-        <v>7.253213978002612</v>
+        <v>6.984542818025049</v>
       </c>
       <c r="N45">
-        <v>0.1726855106721603</v>
+        <v>4.043537801532499</v>
       </c>
       <c r="O45">
-        <v>0.0065830076116025</v>
+        <v>0.044023863402592</v>
       </c>
       <c r="P45">
-        <v>1.080892260092819</v>
+        <v>0.3151354858026847</v>
+      </c>
+      <c r="Q45">
+        <v>0.1119887165021156</v>
+      </c>
+      <c r="R45">
+        <v>0.8817405788049136</v>
+      </c>
+      <c r="S45">
+        <v>1.191475134716996</v>
       </c>
       <c r="U45">
-        <v>2.166334597667929</v>
+        <v>0.0882391306015862</v>
       </c>
       <c r="Z45">
-        <v>3826.718601958101</v>
+        <v>305.8216654384672</v>
+      </c>
+      <c r="AA45">
+        <v>0.0025804412231936</v>
       </c>
       <c r="AD45">
         <v>1</v>
@@ -3263,22 +3314,22 @@
         <v>39</v>
       </c>
       <c r="C46">
-        <v>3.45</v>
+        <v>25.5621</v>
       </c>
       <c r="D46">
-        <v>92.95999999999999</v>
+        <v>100.1299</v>
       </c>
       <c r="F46" t="s">
         <v>42</v>
       </c>
       <c r="H46">
-        <v>1.07</v>
+        <v>63</v>
       </c>
       <c r="I46">
-        <v>5.81</v>
+        <v>471</v>
       </c>
       <c r="J46">
-        <v>12.63</v>
+        <v>8.210000000000001</v>
       </c>
       <c r="L46">
         <v>8.934419422921966</v>
@@ -3352,7 +3403,7 @@
         <v>7.32</v>
       </c>
       <c r="L47">
-        <v>81.92017731391307</v>
+        <v>82.38138755788481</v>
       </c>
       <c r="N47">
         <v>41.95083473870486</v>
@@ -3369,6 +3420,9 @@
       <c r="R47">
         <v>7.241723922548407</v>
       </c>
+      <c r="S47">
+        <v>28.94170130193652</v>
+      </c>
       <c r="U47">
         <v>0.4905584130256302</v>
       </c>
@@ -3376,7 +3430,7 @@
         <v>298.9788398778819</v>
       </c>
       <c r="AA47">
-        <v>28.48049105796478</v>
+        <v>0</v>
       </c>
       <c r="AD47">
         <v>1</v>
@@ -3408,7 +3462,7 @@
         <v>7.32</v>
       </c>
       <c r="L48">
-        <v>54.55722377878762</v>
+        <v>84.49406084661157</v>
       </c>
       <c r="N48">
         <v>42.82165688572165</v>
@@ -3425,6 +3479,9 @@
       <c r="R48">
         <v>7.490214449302519</v>
       </c>
+      <c r="S48">
+        <v>29.93683706782394</v>
+      </c>
       <c r="U48">
         <v>0.4946506625607763</v>
       </c>
@@ -3693,35 +3750,44 @@
       <c r="B53" t="s">
         <v>41</v>
       </c>
+      <c r="C53">
+        <v>25.4829</v>
+      </c>
+      <c r="D53">
+        <v>99.79040000000001</v>
+      </c>
       <c r="F53" t="s">
         <v>42</v>
       </c>
+      <c r="H53">
+        <v>56</v>
+      </c>
       <c r="L53">
-        <v>13.79997500681053</v>
+        <v>20.32098573309655</v>
       </c>
       <c r="N53">
-        <v>4.340643875108097</v>
+        <v>6.603807110893546</v>
       </c>
       <c r="O53">
-        <v>2.304052664060893</v>
+        <v>0.3805801275457725</v>
       </c>
       <c r="P53">
-        <v>3.788113179300364</v>
+        <v>1.730874794151405</v>
       </c>
       <c r="Q53">
-        <v>0.2609308885754584</v>
+        <v>0.5136812411847672</v>
       </c>
       <c r="R53">
-        <v>0.7221528211534458</v>
+        <v>0.4563814282739954</v>
       </c>
       <c r="S53">
-        <v>0.7184906451993549</v>
+        <v>9.882524157281273</v>
       </c>
       <c r="T53">
         <v>0.0288184438040345</v>
       </c>
       <c r="U53">
-        <v>0.6517649104948297</v>
+        <v>0.3790446131929009</v>
       </c>
       <c r="V53">
         <v>143.0495320703036</v>
@@ -3733,10 +3799,10 @@
         <v>0.000589755724635</v>
       </c>
       <c r="Z53">
-        <v>780.082113906727</v>
+        <v>200.0210548478787</v>
       </c>
       <c r="AA53">
-        <v>0.0612854790508492</v>
+        <v>0.001612775764496</v>
       </c>
       <c r="AD53">
         <v>1</v>

</xml_diff>